<commit_message>
Update ONON data - 2026-09-08 08:53:13
</commit_message>
<xml_diff>
--- a/data/ONON_data.xlsx
+++ b/data/ONON_data.xlsx
@@ -10899,7 +10899,7 @@
         <v>19.303448</v>
       </c>
       <c r="L2" t="n">
-        <v>13.501952</v>
+        <v>13.499764</v>
       </c>
       <c r="M2" t="n">
         <v>1.45</v>
@@ -10981,7 +10981,7 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>2026-09-07 03:09:19</t>
+          <t>2026-09-08 08:53:11</t>
         </is>
       </c>
     </row>

</xml_diff>